<commit_message>
adjustment for wip adjustment column excel qty and add report excel
</commit_message>
<xml_diff>
--- a/public/assets/example/template_wip_adjustment_cutting_fabric.xlsx
+++ b/public/assets/example/template_wip_adjustment_cutting_fabric.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\nds_wip\public\assets\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0102262E-32D8-4408-9B3C-F29ACE2075FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B5F228-01C3-41DF-B2BF-7F5761A01065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D854026E-20C0-45F2-B31A-F4C48315BC8B}"/>
   </bookViews>
@@ -53,7 +53,7 @@
     <t>satuan</t>
   </si>
   <si>
-    <t>fabric</t>
+    <t>qty fabric</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
add note in template wip adjustment, and fix import
</commit_message>
<xml_diff>
--- a/public/assets/example/template_wip_adjustment_cutting_fabric.xlsx
+++ b/public/assets/example/template_wip_adjustment_cutting_fabric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\nds_wip\public\assets\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B5F228-01C3-41DF-B2BF-7F5761A01065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B20D194-4508-4157-960F-360D870462DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D854026E-20C0-45F2-B31A-F4C48315BC8B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>tgl_saldo</t>
   </si>
@@ -54,13 +54,54 @@
   </si>
   <si>
     <t>qty fabric</t>
+  </si>
+  <si>
+    <t>SMT/0426/029</t>
+  </si>
+  <si>
+    <t>F260713516</t>
+  </si>
+  <si>
+    <t>METER</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">*Baris pertama </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>jangan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dihapus/diubah</t>
+    </r>
+  </si>
+  <si>
+    <t>*Baris kedua hanya data contoh, silahkan hapus lalu isi kembali dengan data yang asli</t>
+  </si>
+  <si>
+    <t>*Pastikan diisi dengan sesuai kolomnya</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -75,8 +116,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -86,6 +135,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -105,9 +160,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -656,7 +713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D1A05E2-1099-486A-ABC2-C2A526A6CF74}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
@@ -665,9 +722,10 @@
     <col min="4" max="4" width="13.42578125" customWidth="1"/>
     <col min="5" max="5" width="9.5703125" customWidth="1"/>
     <col min="6" max="6" width="11.5703125" customWidth="1"/>
+    <col min="7" max="7" width="80.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -685,9 +743,41 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>46234</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>61903</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G3" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adjustment font excel to calibri
</commit_message>
<xml_diff>
--- a/public/assets/example/template_wip_adjustment_cutting_fabric.xlsx
+++ b/public/assets/example/template_wip_adjustment_cutting_fabric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\nds_wip\public\assets\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B20D194-4508-4157-960F-360D870462DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{371991EC-2F15-4018-B0C1-78BA2F191312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D854026E-20C0-45F2-B31A-F4C48315BC8B}"/>
   </bookViews>
@@ -65,6 +65,12 @@
     <t>METER</t>
   </si>
   <si>
+    <t>*Baris kedua hanya data contoh, silahkan hapus lalu isi kembali dengan data yang asli</t>
+  </si>
+  <si>
+    <t>*Pastikan diisi dengan sesuai kolomnya</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">*Baris pertama </t>
     </r>
@@ -73,9 +79,8 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </rPr>
       <t>jangan</t>
     </r>
@@ -83,25 +88,18 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> dihapus/diubah</t>
     </r>
-  </si>
-  <si>
-    <t>*Baris kedua hanya data contoh, silahkan hapus lalu isi kembali dengan data yang asli</t>
-  </si>
-  <si>
-    <t>*Pastikan diisi dengan sesuai kolomnya</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,12 +115,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -160,11 +163,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -716,13 +720,14 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" customWidth="1"/>
-    <col min="7" max="7" width="80.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="80.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -744,36 +749,36 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
+      <c r="G1" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>46234</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3">
         <v>61903</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>1</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>10</v>
+      <c r="G2" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G3" s="3" t="s">
-        <v>11</v>
+      <c r="G3" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>